<commit_message>
feat(footer): update mobile bottom contact action sheet and simplify bottom nav
</commit_message>
<xml_diff>
--- a/DailyXeDien_Rebuild_Planv1.1_formatted.xlsx
+++ b/DailyXeDien_Rebuild_Planv1.1_formatted.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,8 +97,15 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Be Vietnam Pro"/>
+      <b val="1"/>
+      <color rgb="00F57F17"/>
+      <sz val="10"/>
+    </font>
+    <font/>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -151,6 +158,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="000D47A1"/>
         <bgColor rgb="000D47A1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFDE7"/>
+        <bgColor rgb="00FFFDE7"/>
       </patternFill>
     </fill>
   </fills>
@@ -239,7 +252,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -331,6 +344,55 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -755,9 +817,9 @@
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
       <c r="D1" s="2" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="4" t="n"/>
-      <c r="G1" s="4" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="3" t="n"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
@@ -1217,107 +1279,107 @@
       </c>
     </row>
     <row r="15" ht="35" customHeight="1">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="15" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>Tháng 3 (T8)</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Performance Optimization</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>15/08</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>28/08</t>
         </is>
       </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Tối ưu Core Web Vitals: LCP (WebP, fetchpriority), Schema (Breadcrumb, Article).</t>
+      <c r="F15" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="G15" s="17" t="inlineStr">
+        <is>
+          <t>Tối ưu Core Web Vitals: LCP (WebP, fetchpriority), LiteSpeed cache, DB optimization. Hoàn thành: 14/07/2026</t>
         </is>
       </c>
     </row>
     <row r="16" ht="35" customHeight="1">
-      <c r="A16" s="9" t="n">
+      <c r="A16" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
         <is>
           <t>Tháng 3 (T8)</t>
         </is>
       </c>
-      <c r="C16" s="10" t="inlineStr">
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t>SEO: LCP (WebP/fetchpriority) + Schema (Breadcrumb, Article)</t>
         </is>
       </c>
-      <c r="D16" s="10" t="inlineStr">
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>15/08</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>28/08</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="G16" s="10" t="inlineStr">
-        <is>
-          <t>Tối ưu hiệu suất: cấu hình LiteSpeed cache, tối ưu database, lazy load.</t>
+      <c r="F16" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="G16" s="17" t="inlineStr">
+        <is>
+          <t>Tối ưu hiệu suất LCP, tích hợp Schema markup (Product, Article, Breadcrumb, LocalBusiness). Hoàn thành: 17/07/2026</t>
         </is>
       </c>
     </row>
     <row r="17" ht="35" customHeight="1">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="15" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
         <is>
           <t>Tháng 3 (T8)</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>SEO Technical fixes</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>22/08</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>31/08</t>
         </is>
       </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Sửa lỗi SEO kỹ thuật: schema markup, robots.txt, sitemap XML đúng chuẩn.</t>
+      <c r="F17" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>Chuyển đổi Rank Math, tạo bản đồ redirect 301, redesign trang 404. Hoàn thành: 18/07/2026</t>
         </is>
       </c>
     </row>
@@ -1502,12 +1564,6 @@
           <t>SPL Theme là theme WordPress custom tự code hoàn toàn, KHÔNG dùng Flatsome UX Builder. Code trực tiếp PHP + SCSS + Vite giúp tăng hiệu suất gấp 2-3x, giảm ~2MB JS/CSS builder, đạt PageSpeed cao hơn.</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="13" t="n"/>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="13" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
@@ -1515,12 +1571,6 @@
           <t>⚠️ LƯU Ý: Plan này có thể được thay đổi, cập nhật trong quá trình triển khai tùy theo tình hình thực tế.</t>
         </is>
       </c>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="14" t="n"/>
-      <c r="E26" s="14" t="n"/>
-      <c r="F26" s="14" t="n"/>
-      <c r="G26" s="14" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="$A$2:$G$22"/>
@@ -1539,7 +1589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2827,739 +2877,1607 @@
       </c>
     </row>
     <row r="38" ht="30" customHeight="1">
-      <c r="A38" s="9" t="n">
+      <c r="A38" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="B38" s="27" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
         <is>
           <t>T3</t>
         </is>
       </c>
-      <c r="C38" s="27" t="inlineStr">
+      <c r="C38" s="16" t="inlineStr">
         <is>
           <t>Tuần 3</t>
         </is>
       </c>
-      <c r="D38" s="10" t="inlineStr">
+      <c r="D38" s="17" t="inlineStr">
         <is>
           <t>Hiệu suất: Cấu hình LiteSpeed cache</t>
         </is>
       </c>
-      <c r="E38" s="12" t="inlineStr">
+      <c r="E38" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F38" s="35" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>Thiết lập LiteSpeed cache trên server staging/production. Hoàn thành: 14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="15" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>Hiệu suất: Tối ưu database</t>
+        </is>
+      </c>
+      <c r="E39" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F39" s="36" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G39" s="17" t="inlineStr">
+        <is>
+          <t>Xóa bản nháp cũ, transients hết hạn, tối ưu DB. Hoàn thành: 14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="15" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>Hiệu suất: Tải trước hero + fonts</t>
+        </is>
+      </c>
+      <c r="E40" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F40" s="36" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G40" s="17" t="inlineStr">
+        <is>
+          <t>Tải trước hero image WebP (fetchpriority), font Be Vietnam Pro. Hoàn thành: 14/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="15" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>SEO: Gỡ Yoast, thống nhất Rank Math</t>
+        </is>
+      </c>
+      <c r="E41" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F41" s="35" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G41" s="17" t="inlineStr">
+        <is>
+          <t>Thống nhất Rank Math SEO, xuất sitemap XML, robots.txt. Hoàn thành: 15/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="15" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>SEO: Schema markup cấu trúc</t>
+        </is>
+      </c>
+      <c r="E42" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F42" s="36" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G42" s="17" t="inlineStr">
+        <is>
+          <t>Tích hợp Schema Product, LocalBusiness, Breadcrumb, Article. Hoàn thành: 17/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="15" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>SEO: Bản đồ redirect 301</t>
+        </is>
+      </c>
+      <c r="E43" s="34" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F43" s="35" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G43" s="17" t="inlineStr">
+        <is>
+          <t>Tạo bản đồ redirect 301 đầy đủ cho tất cả URL cũ. Hoàn thành: 18/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>SEO: Redesign trang 404</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F44" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G44" s="17" t="inlineStr">
+        <is>
+          <t>Thiết kế lại trang 404 theo chuẩn htmlmau &amp; theme 404.php. Hoàn thành: 18/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="15" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>Layout: Fix spacing mobile homepage</t>
+        </is>
+      </c>
+      <c r="E45" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F45" s="8" t="inlineStr">
+        <is>
+          <t>🟢 Thấp</t>
+        </is>
+      </c>
+      <c r="G45" s="17" t="inlineStr">
+        <is>
+          <t>Sửa lề và khoảng cách mobile trên homepage. Hoàn thành: 18/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1">
+      <c r="A46" s="15" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>Layout: Fix breadcrumb mobile single page</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>🟢 Thấp</t>
+        </is>
+      </c>
+      <c r="G46" s="17" t="inlineStr">
+        <is>
+          <t>Tối ưu hiển thị breadcrumb trên mobile trong single.php. Hoàn thành: 18/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1">
+      <c r="A47" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>Layout: Fix mũi tên slider video</t>
+        </is>
+      </c>
+      <c r="E47" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F47" s="8" t="inlineStr">
+        <is>
+          <t>🟢 Thấp</t>
+        </is>
+      </c>
+      <c r="G47" s="17" t="inlineStr">
+        <is>
+          <t>Fix mũi tên chuyển slide video SVG trong media-reviews.php. Hoàn thành: 18/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1">
+      <c r="A48" s="15" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C48" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>Layout: Cập nhật footer text &amp; logo BCT</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>🟢 Thấp</t>
+        </is>
+      </c>
+      <c r="G48" s="17" t="inlineStr">
+        <is>
+          <t>Cập nhật thông tin footer và logo Bộ Công Thương SVG. Hoàn thành: 18/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1">
+      <c r="A49" s="15" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="C49" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>Portfolio Gallery: Tạo CPT &amp; Import/Export</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F49" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G49" s="17" t="inlineStr">
+        <is>
+          <t>Tạo CPT portfolio_gallery + script export/import dữ liệu. Hoàn thành: 26/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1">
+      <c r="A50" s="15" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C50" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 1</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>Portfolio Gallery: Homepage Tab Section</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F50" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G50" s="17" t="inlineStr">
+        <is>
+          <t>Tạo section tab Portfolio Gallery trên trang chủ. Hoàn thành: 26/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="15" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C51" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 1</t>
+        </is>
+      </c>
+      <c r="D51" s="17" t="inlineStr">
+        <is>
+          <t>Portfolio Gallery: Page Cache &amp; Bug Fixes</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>🟢 Thấp</t>
+        </is>
+      </c>
+      <c r="G51" s="17" t="inlineStr">
+        <is>
+          <t>Fix lỗi hiển thị và tích hợp page cache. Hoàn thành: 26/06/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="30" customHeight="1">
+      <c r="A52" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C52" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 1</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>Giao diện: Trang Hợp Tác (Cooperation)</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F52" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G52" s="17" t="inlineStr">
+        <is>
+          <t>Code template page-hop-tac.php + CSS styling chuẩn htmlmau. Hoàn thành: 04/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="15" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C53" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 1</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>Giao diện: Single Product JS interactions</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F53" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>Thêm JS QuickView, gallery zoom, tabs tương tác trang sản phẩm. Hoàn thành: 04/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="30" customHeight="1">
+      <c r="A54" s="15" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C54" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 2</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Giao diện: Blog templates &amp; Table of Contents</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F54" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>Code template bài viết blog + tự động tạo mục lục TOC. Hoàn thành: 08/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="15" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C55" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 2</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>Giao diện: WC Cart &amp; Checkout layout polish</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F55" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>Tối ưu giao diện giỏ hàng và thanh toán WooCommerce. Hoàn thành: 13/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="30" customHeight="1">
+      <c r="A56" s="15" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>Mobile Bottom Menu 6 nút</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F56" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G56" s="17" t="inlineStr">
+        <is>
+          <t>Tạo menu bottom mobile: Trang chủ, Danh mục, Tin tức, Đại lý, Liên hệ, Giỏ hàng. Hoàn thành: 17/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
+      <c r="A57" s="15" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C57" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>Slide-up Panel Danh mục sản phẩm</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F57" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>Slide-up Panel 2 cột cho Danh mục SP (truy vấn WC categories động). Hoàn thành: 17/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="15" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C58" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>Slide-up Panel Tin tức</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F58" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G58" s="17" t="inlineStr">
+        <is>
+          <t>Slide-up Panel 2 cột Tin tức (truy vấn danh mục bài viết, 4 bài mới nhất). Hoàn thành: 17/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="30" customHeight="1">
+      <c r="A59" s="15" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C59" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>Slide-up Panel Đại lý</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F59" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G59" s="17" t="inlineStr">
+        <is>
+          <t>Slide-up Panel Đại lý (sắp xếp tỉnh thành theo số đại lý, TP.HCM lên đầu). Hoàn thành: 17/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="30" customHeight="1">
+      <c r="A60" s="15" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C60" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>Slide-up Panel Liên hệ</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>🟢 Thấp</t>
+        </is>
+      </c>
+      <c r="G60" s="17" t="inlineStr">
+        <is>
+          <t>Slide-up Panel Liên hệ (Hotline, Zalo, Form link). Hoàn thành: 17/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="30" customHeight="1">
+      <c r="A61" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C61" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>ACF Options quản lý Mobile Menu</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F61" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G61" s="17" t="inlineStr">
+        <is>
+          <t>Đăng ký ACF Options bật/tắt danh mục hiển thị trên menu bottom. Hoàn thành: 17/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="30" customHeight="1">
+      <c r="A62" s="15" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C62" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="inlineStr">
+        <is>
+          <t>Fix giao diện Card &amp; Swiper Mobile Panel</t>
+        </is>
+      </c>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F62" s="8" t="inlineStr">
+        <is>
+          <t>🟢 Thấp</t>
+        </is>
+      </c>
+      <c r="G62" s="17" t="inlineStr">
+        <is>
+          <t>Fix Card hover/active, text giá WC, đè mũi tên Swiper. Hoàn thành: 17/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="30" customHeight="1">
+      <c r="A63" s="15" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
+        <is>
+          <t>Giao diện: PC Header Mega Menu Dynamic</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F63" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>Chuyển đổi danh mục hover sản phẩm động trên PC Mega Menu. Hoàn thành: 22/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="30" customHeight="1">
+      <c r="A64" s="15" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C64" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D64" s="17" t="inlineStr">
+        <is>
+          <t>UX/UI: Responsive tất cả inner pages</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F64" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G64" s="17" t="inlineStr">
+        <is>
+          <t>Tối ưu responsive cho tất cả trang nội dung trên mobile/tablet. Hoàn thành: 22/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="30" customHeight="1">
+      <c r="A65" s="15" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C65" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D65" s="17" t="inlineStr">
+        <is>
+          <t>Giao diện: Trang Hợp Tác Bluera mở rộng</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F65" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G65" s="17" t="inlineStr">
+        <is>
+          <t>Mở rộng trang Cooperation + Header UI fixes. Hoàn thành: 25/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="30" customHeight="1">
+      <c r="A66" s="15" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C66" s="16" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D66" s="17" t="inlineStr">
+        <is>
+          <t>Giao diện: Trang Giới Thiệu (About)</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
+        </is>
+      </c>
+      <c r="F66" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G66" s="17" t="inlineStr">
+        <is>
+          <t>Cập nhật trang About (Hero, CEO Message, CTA) chuẩn htmlmau. Hoàn thành: 27/07/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="9" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C67" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 1</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>Xác nhận GSC: quyền sở hữu, sitemap, phạm vi</t>
+        </is>
+      </c>
+      <c r="E67" s="12" t="inlineStr">
         <is>
           <t>⬜ Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="F38" s="18" t="inlineStr">
+      <c r="F67" s="18" t="inlineStr">
         <is>
           <t>🔴 Cao</t>
         </is>
       </c>
-      <c r="G38" s="10" t="inlineStr">
-        <is>
-          <t>Thiết lập cache trên server production cho tốc độ tối đa</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="30" customHeight="1">
-      <c r="A39" s="28" t="n">
-        <v>37</v>
-      </c>
-      <c r="B39" s="29" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="C39" s="29" t="inlineStr">
+      <c r="G67" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra Google Search Console: 0 lỗi index coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="30" customHeight="1">
+      <c r="A68" s="9" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C68" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 1</t>
+        </is>
+      </c>
+      <c r="D68" s="10" t="inlineStr">
+        <is>
+          <t>Xác nhận GA4: theo dõi, sự kiện thương mại</t>
+        </is>
+      </c>
+      <c r="E68" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F68" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G68" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra GA4 events: purchase, add_to_cart hoạt động đúng</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="30" customHeight="1">
+      <c r="A69" s="9" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C69" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 1</t>
+        </is>
+      </c>
+      <c r="D69" s="10" t="inlineStr">
+        <is>
+          <t>Xác nhận Google Ads: chuyển đổi, remarketing</t>
+        </is>
+      </c>
+      <c r="E69" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F69" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G69" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra conversion tag, remarketing tag, Merchant Center</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="9" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C70" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 1</t>
+        </is>
+      </c>
+      <c r="D70" s="10" t="inlineStr">
+        <is>
+          <t>Xác nhận sự kiện Facebook Pixel</t>
+        </is>
+      </c>
+      <c r="E70" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F70" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G70" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra FB Pixel events qua TrackingPixels.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="30" customHeight="1">
+      <c r="A71" s="9" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C71" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 2</t>
+        </is>
+      </c>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>Xác nhận thanh toán BaoKim E2E</t>
+        </is>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F71" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G71" s="10" t="inlineStr">
+        <is>
+          <t>Test luồng checkout đến thanh toán đến xác nhận đơn hàng</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="30" customHeight="1">
+      <c r="A72" s="9" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C72" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 2</t>
+        </is>
+      </c>
+      <c r="D72" s="10" t="inlineStr">
+        <is>
+          <t>Xác nhận hiển thị cửa hàng DevVN Stores</t>
+        </is>
+      </c>
+      <c r="E72" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F72" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G72" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra bản đồ cửa hàng đại lý hiển thị đúng</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="30" customHeight="1">
+      <c r="A73" s="9" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C73" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 2</t>
+        </is>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>Xác nhận email qua Fluent SMTP</t>
+        </is>
+      </c>
+      <c r="E73" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F73" s="50" t="inlineStr">
+        <is>
+          <t>🟡 TB</t>
+        </is>
+      </c>
+      <c r="G73" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra email giao dịch gửi thành công qua SMTP</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="9" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C74" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 2</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>QA: Quét toàn site (0 link hỏng)</t>
+        </is>
+      </c>
+      <c r="E74" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F74" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G74" s="10" t="inlineStr">
+        <is>
+          <t>Dùng Screaming Frog quét tìm broken links, sửa hết</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="30" customHeight="1">
+      <c r="A75" s="9" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C75" s="27" t="inlineStr">
         <is>
           <t>Tuần 3</t>
         </is>
       </c>
-      <c r="D39" s="30" t="inlineStr">
-        <is>
-          <t>Hiệu suất: Tối ưu database</t>
-        </is>
-      </c>
-      <c r="E39" s="31" t="inlineStr">
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>QA: Test mobile (3+ thiết bị)</t>
+        </is>
+      </c>
+      <c r="E75" s="12" t="inlineStr">
         <is>
           <t>⬜ Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="F39" s="26" t="inlineStr">
+      <c r="F75" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G75" s="10" t="inlineStr">
+        <is>
+          <t>Kiểm tra giao diện trên ít nhất 3 thiết bị mobile khác nhau</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="30" customHeight="1">
+      <c r="A76" s="9" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C76" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>QA: Kiểm tra schema markup</t>
+        </is>
+      </c>
+      <c r="E76" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F76" s="50" t="inlineStr">
         <is>
           <t>🟡 TB</t>
         </is>
       </c>
-      <c r="G39" s="30" t="inlineStr">
-        <is>
-          <t>Xóa bản nháp cũ, transients hết hạn, tối ưu bảng DB</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="9" t="n">
-        <v>38</v>
-      </c>
-      <c r="B40" s="27" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="C40" s="27" t="inlineStr">
+      <c r="G76" s="10" t="inlineStr">
+        <is>
+          <t>Dùng Google Rich Results Test xác nhận schema hợp lệ</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="9" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C77" s="27" t="inlineStr">
         <is>
           <t>Tuần 3</t>
         </is>
       </c>
-      <c r="D40" s="10" t="inlineStr">
-        <is>
-          <t>Hiệu suất: Tải trước hero + fonts</t>
-        </is>
-      </c>
-      <c r="E40" s="12" t="inlineStr">
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>QA: PageSpeed ≥75 mobile, ≥92 desktop</t>
+        </is>
+      </c>
+      <c r="E77" s="12" t="inlineStr">
         <is>
           <t>⬜ Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="F40" s="19" t="inlineStr">
+      <c r="F77" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G77" s="10" t="inlineStr">
+        <is>
+          <t>Đảm bảo đạt điểm tốc độ mục tiêu trên PageSpeed Insights</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="9" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C78" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 3</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>Triển khai: Tải lên theme + plugins</t>
+        </is>
+      </c>
+      <c r="E78" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F78" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G78" s="10" t="inlineStr">
+        <is>
+          <t>Deploy theo từng bước (staged rollout), không deploy 1 lần</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="9" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C79" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>Triển khai: Tắt plugin cũ (5/đợt)</t>
+        </is>
+      </c>
+      <c r="E79" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F79" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G79" s="10" t="inlineStr">
+        <is>
+          <t>Tắt từng nhóm 5 plugin, kiểm tra sau mỗi đợt</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="9" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C80" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D80" s="10" t="inlineStr">
+        <is>
+          <t>Giám sát: GSC hàng ngày 14 ngày</t>
+        </is>
+      </c>
+      <c r="E80" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="inlineStr">
+        <is>
+          <t>🔴 Cao</t>
+        </is>
+      </c>
+      <c r="G80" s="10" t="inlineStr">
+        <is>
+          <t>Theo dõi GSC mỗi ngày, fix lỗi 404 ngay khi phát hiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" s="27" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C81" s="27" t="inlineStr">
+        <is>
+          <t>Tuần 4</t>
+        </is>
+      </c>
+      <c r="D81" s="10" t="inlineStr">
+        <is>
+          <t>Giám sát: So sánh traffic GA4</t>
+        </is>
+      </c>
+      <c r="E81" s="12" t="inlineStr">
+        <is>
+          <t>⬜ Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="F81" s="50" t="inlineStr">
         <is>
           <t>🟡 TB</t>
         </is>
       </c>
-      <c r="G40" s="10" t="inlineStr">
-        <is>
-          <t>Dùng fetchpriority, preconnect để tải trước tài nguyên quan trọng</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" s="32" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="C41" s="32" t="inlineStr">
-        <is>
-          <t>Tuần 4</t>
-        </is>
-      </c>
-      <c r="D41" s="7" t="inlineStr">
-        <is>
-          <t>SEO: Gỡ Yoast, thống nhất Rank Math</t>
-        </is>
-      </c>
-      <c r="E41" s="11" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F41" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>Dùng 1 plugin SEO duy nhất, cập nhật robots.txt và sitemap</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="9" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" s="27" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="C42" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 4</t>
-        </is>
-      </c>
-      <c r="D42" s="10" t="inlineStr">
-        <is>
-          <t>SEO: Schema markup cấu trúc</t>
-        </is>
-      </c>
-      <c r="E42" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F42" s="19" t="inlineStr">
-        <is>
-          <t>🟡 TB</t>
-        </is>
-      </c>
-      <c r="G42" s="10" t="inlineStr">
-        <is>
-          <t>Thêm dữ liệu có cấu trúc Product, Organization, LocalBusiness</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="30" customHeight="1">
-      <c r="A43" s="6" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" s="32" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="C43" s="32" t="inlineStr">
-        <is>
-          <t>Tuần 4</t>
-        </is>
-      </c>
-      <c r="D43" s="7" t="inlineStr">
-        <is>
-          <t>SEO: Bản đồ redirect 301</t>
-        </is>
-      </c>
-      <c r="E43" s="11" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F43" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>Tạo danh sách redirect 301 đầy đủ bằng Rank Math Redirections</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="30" customHeight="1">
-      <c r="A44" s="9" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" s="27" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C44" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 1</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>Xác nhận GSC: quyền sở hữu, sitemap, phạm vi</t>
-        </is>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F44" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G44" s="10" t="inlineStr">
-        <is>
-          <t>Kiểm tra Google Search Console: 0 lỗi index coverage</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="30" customHeight="1">
-      <c r="A45" s="28" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" s="29" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C45" s="29" t="inlineStr">
-        <is>
-          <t>Tuần 1</t>
-        </is>
-      </c>
-      <c r="D45" s="30" t="inlineStr">
-        <is>
-          <t>Xác nhận GA4: theo dõi, sự kiện thương mại</t>
-        </is>
-      </c>
-      <c r="E45" s="31" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F45" s="24" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G45" s="30" t="inlineStr">
-        <is>
-          <t>Kiểm tra GA4 events: purchase, add_to_cart hoạt động đúng</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="9" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" s="27" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C46" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 1</t>
-        </is>
-      </c>
-      <c r="D46" s="10" t="inlineStr">
-        <is>
-          <t>Xác nhận Google Ads: chuyển đổi, remarketing</t>
-        </is>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F46" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G46" s="10" t="inlineStr">
-        <is>
-          <t>Kiểm tra conversion tag, remarketing tag, Merchant Center</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="6" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C47" s="32" t="inlineStr">
-        <is>
-          <t>Tuần 1</t>
-        </is>
-      </c>
-      <c r="D47" s="7" t="inlineStr">
-        <is>
-          <t>Xác nhận sự kiện Facebook Pixel</t>
-        </is>
-      </c>
-      <c r="E47" s="11" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F47" s="19" t="inlineStr">
-        <is>
-          <t>🟡 TB</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>Kiểm tra FB Pixel events qua TrackingPixels.php</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="9" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" s="27" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C48" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 2</t>
-        </is>
-      </c>
-      <c r="D48" s="10" t="inlineStr">
-        <is>
-          <t>Xác nhận thanh toán BaoKim E2E</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F48" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G48" s="10" t="inlineStr">
-        <is>
-          <t>Test luồng checkout đến thanh toán đến xác nhận đơn hàng</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="28" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" s="29" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C49" s="29" t="inlineStr">
-        <is>
-          <t>Tuần 2</t>
-        </is>
-      </c>
-      <c r="D49" s="30" t="inlineStr">
-        <is>
-          <t>Xác nhận hiển thị cửa hàng DevVN Stores</t>
-        </is>
-      </c>
-      <c r="E49" s="31" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F49" s="26" t="inlineStr">
-        <is>
-          <t>🟡 TB</t>
-        </is>
-      </c>
-      <c r="G49" s="30" t="inlineStr">
-        <is>
-          <t>Kiểm tra bản đồ cửa hàng đại lý hiển thị đúng</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="9" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" s="27" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C50" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 2</t>
-        </is>
-      </c>
-      <c r="D50" s="10" t="inlineStr">
-        <is>
-          <t>Xác nhận email qua Fluent SMTP</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F50" s="19" t="inlineStr">
-        <is>
-          <t>🟡 TB</t>
-        </is>
-      </c>
-      <c r="G50" s="10" t="inlineStr">
-        <is>
-          <t>Kiểm tra email giao dịch gửi thành công qua SMTP</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="30" customHeight="1">
-      <c r="A51" s="6" t="n">
-        <v>49</v>
-      </c>
-      <c r="B51" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C51" s="32" t="inlineStr">
-        <is>
-          <t>Tuần 2</t>
-        </is>
-      </c>
-      <c r="D51" s="7" t="inlineStr">
-        <is>
-          <t>QA: Quét toàn site (0 link hỏng)</t>
-        </is>
-      </c>
-      <c r="E51" s="11" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F51" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>Dùng Screaming Frog quét tìm broken links, sửa hết</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="9" t="n">
-        <v>50</v>
-      </c>
-      <c r="B52" s="27" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C52" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 3</t>
-        </is>
-      </c>
-      <c r="D52" s="10" t="inlineStr">
-        <is>
-          <t>QA: Test mobile (3+ thiết bị)</t>
-        </is>
-      </c>
-      <c r="E52" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F52" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>Kiểm tra giao diện trên ít nhất 3 thiết bị mobile khác nhau</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="28" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" s="29" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C53" s="29" t="inlineStr">
-        <is>
-          <t>Tuần 3</t>
-        </is>
-      </c>
-      <c r="D53" s="30" t="inlineStr">
-        <is>
-          <t>QA: Kiểm tra schema markup</t>
-        </is>
-      </c>
-      <c r="E53" s="31" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F53" s="26" t="inlineStr">
-        <is>
-          <t>🟡 TB</t>
-        </is>
-      </c>
-      <c r="G53" s="30" t="inlineStr">
-        <is>
-          <t>Dùng Google Rich Results Test xác nhận schema hợp lệ</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="9" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" s="27" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C54" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 3</t>
-        </is>
-      </c>
-      <c r="D54" s="10" t="inlineStr">
-        <is>
-          <t>QA: PageSpeed ≥75 mobile, ≥92 desktop</t>
-        </is>
-      </c>
-      <c r="E54" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F54" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G54" s="10" t="inlineStr">
-        <is>
-          <t>Đảm bảo đạt điểm tốc độ mục tiêu trên PageSpeed Insights</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="6" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" s="32" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C55" s="32" t="inlineStr">
-        <is>
-          <t>Tuần 3</t>
-        </is>
-      </c>
-      <c r="D55" s="7" t="inlineStr">
-        <is>
-          <t>Triển khai: Tải lên theme + plugins</t>
-        </is>
-      </c>
-      <c r="E55" s="11" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F55" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>Deploy theo từng bước (staged rollout), không deploy 1 lần</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="9" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" s="27" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C56" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 4</t>
-        </is>
-      </c>
-      <c r="D56" s="10" t="inlineStr">
-        <is>
-          <t>Triển khai: Tắt plugin cũ (5/đợt)</t>
-        </is>
-      </c>
-      <c r="E56" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F56" s="18" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G56" s="10" t="inlineStr">
-        <is>
-          <t>Tắt từng nhóm 5 plugin, kiểm tra sau mỗi đợt</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="30" customHeight="1">
-      <c r="A57" s="28" t="n">
-        <v>55</v>
-      </c>
-      <c r="B57" s="29" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C57" s="29" t="inlineStr">
-        <is>
-          <t>Tuần 4</t>
-        </is>
-      </c>
-      <c r="D57" s="30" t="inlineStr">
-        <is>
-          <t>Giám sát: GSC hàng ngày 14 ngày</t>
-        </is>
-      </c>
-      <c r="E57" s="31" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F57" s="24" t="inlineStr">
-        <is>
-          <t>🔴 Cao</t>
-        </is>
-      </c>
-      <c r="G57" s="30" t="inlineStr">
-        <is>
-          <t>Theo dõi GSC mỗi ngày, fix lỗi 404 ngay khi phát hiện</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="30" customHeight="1">
-      <c r="A58" s="9" t="n">
-        <v>56</v>
-      </c>
-      <c r="B58" s="27" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="C58" s="27" t="inlineStr">
-        <is>
-          <t>Tuần 4</t>
-        </is>
-      </c>
-      <c r="D58" s="10" t="inlineStr">
-        <is>
-          <t>Giám sát: So sánh traffic GA4</t>
-        </is>
-      </c>
-      <c r="E58" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="F58" s="19" t="inlineStr">
-        <is>
-          <t>🟡 TB</t>
-        </is>
-      </c>
-      <c r="G58" s="10" t="inlineStr">
+      <c r="G81" s="10" t="inlineStr">
         <is>
           <t>So sánh lượng truy cập GA4 với tháng trước để đánh giá</t>
         </is>
       </c>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="49" t="n"/>
+      <c r="B82" s="49" t="n"/>
+      <c r="C82" s="49" t="n"/>
+      <c r="D82" s="49" t="n"/>
+      <c r="E82" s="49" t="n"/>
+      <c r="F82" s="49" t="n"/>
+      <c r="G82" s="49" t="n"/>
+    </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="49" t="n"/>
+      <c r="B83" s="49" t="n"/>
+      <c r="C83" s="49" t="n"/>
+      <c r="D83" s="49" t="n"/>
+      <c r="E83" s="49" t="n"/>
+      <c r="F83" s="49" t="n"/>
+      <c r="G83" s="49" t="n"/>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="49" t="n"/>
+      <c r="B84" s="49" t="n"/>
+      <c r="C84" s="49" t="n"/>
+      <c r="D84" s="49" t="n"/>
+      <c r="E84" s="49" t="n"/>
+      <c r="F84" s="49" t="n"/>
+      <c r="G84" s="49" t="n"/>
+    </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="49" t="n"/>
+      <c r="B85" s="49" t="n"/>
+      <c r="C85" s="49" t="n"/>
+      <c r="D85" s="49" t="n"/>
+      <c r="E85" s="49" t="n"/>
+      <c r="F85" s="49" t="n"/>
+      <c r="G85" s="49" t="n"/>
+    </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="49" t="n"/>
+      <c r="B86" s="49" t="n"/>
+      <c r="C86" s="49" t="n"/>
+      <c r="D86" s="49" t="n"/>
+      <c r="E86" s="49" t="n"/>
+      <c r="F86" s="49" t="n"/>
+      <c r="G86" s="49" t="n"/>
+    </row>
+    <row r="87" ht="30" customHeight="1">
+      <c r="A87" s="49" t="n"/>
+      <c r="B87" s="49" t="n"/>
+      <c r="C87" s="49" t="n"/>
+      <c r="D87" s="49" t="n"/>
+      <c r="E87" s="49" t="n"/>
+      <c r="F87" s="49" t="n"/>
+      <c r="G87" s="49" t="n"/>
+    </row>
+    <row r="88" ht="30" customHeight="1">
+      <c r="A88" s="49" t="n"/>
+      <c r="B88" s="49" t="n"/>
+      <c r="C88" s="49" t="n"/>
+      <c r="D88" s="49" t="n"/>
+      <c r="E88" s="49" t="n"/>
+      <c r="F88" s="49" t="n"/>
+      <c r="G88" s="49" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="$A$2:$G$58"/>
@@ -3576,7 +4494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3593,11 +4511,11 @@
           <t>🔌 PLUGIN MAPPING: CŨ → MỚI (50 → 13)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -3650,9 +4568,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E3" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
@@ -3680,9 +4598,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E4" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E4" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr">
@@ -3710,9 +4628,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E5" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -3740,9 +4658,9 @@
           <t>Polylang FREE + PolylangBridge</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E6" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F6" s="10" t="inlineStr">
@@ -3770,9 +4688,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -3800,9 +4718,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E8" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr">
@@ -3830,9 +4748,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E9" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -3860,9 +4778,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E10" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -3890,9 +4808,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -3920,9 +4838,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E12" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -3950,9 +4868,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E13" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -3980,9 +4898,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E14" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr">
@@ -4010,9 +4928,9 @@
           <t>Fluent SMTP</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E15" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -4040,9 +4958,9 @@
           <t>SPL-A plugin</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E16" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
@@ -4070,9 +4988,9 @@
           <t>SPL-A plugin</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E17" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -4100,9 +5018,9 @@
           <t>SPL-A plugin</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E18" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
@@ -4130,9 +5048,9 @@
           <t>SPL WooCommerce/Swatches</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E19" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -4160,9 +5078,9 @@
           <t>SPL WooCommerce/Gallery</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E20" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
@@ -4190,9 +5108,9 @@
           <t>SPL Features/Optimizer</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E21" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -4220,9 +5138,9 @@
           <t>SPL Features/Optimizer</t>
         </is>
       </c>
-      <c r="E22" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E22" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -4250,9 +5168,9 @@
           <t>GA4 via Site Kit</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E23" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -4280,9 +5198,9 @@
           <t>SPL Modules/PostView</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E24" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F24" s="10" t="inlineStr">
@@ -4310,9 +5228,9 @@
           <t>spl-child TrackingPixels</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E25" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -4340,9 +5258,9 @@
           <t>spl-child LoanShortcode</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E26" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -4370,9 +5288,9 @@
           <t>spl-child SeasonalModule</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E27" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -4400,9 +5318,9 @@
           <t>Code shortcode child</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E28" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr">
@@ -4430,9 +5348,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E29" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -4460,9 +5378,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E30" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E30" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F30" s="10" t="inlineStr">
@@ -4490,9 +5408,9 @@
           <t>SPL ShortcodeLoader</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E31" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
@@ -4520,9 +5438,9 @@
           <t>ACF Repeater (TSKT)</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E32" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr">
@@ -4550,9 +5468,9 @@
           <t>Code trong child</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E33" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -4580,9 +5498,9 @@
           <t>WC product tab code</t>
         </is>
       </c>
-      <c r="E34" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E34" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F34" s="10" t="inlineStr">
@@ -4610,9 +5528,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E35" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -4670,9 +5588,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E37" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
@@ -4700,9 +5618,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E38" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E38" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F38" s="10" t="inlineStr">
@@ -4730,9 +5648,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E39" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
@@ -4760,9 +5678,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E40" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E40" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F40" s="10" t="inlineStr">
@@ -4790,9 +5708,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E41" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
@@ -4820,9 +5738,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E42" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E42" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F42" s="10" t="inlineStr">
@@ -4850,9 +5768,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E43" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
@@ -4880,9 +5798,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E44" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E44" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr">
@@ -4910,9 +5828,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E45" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
@@ -4940,9 +5858,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E46" s="10" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E46" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr">
@@ -4970,9 +5888,9 @@
           <t>PolylangBridge module</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E47" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
@@ -4981,58 +5899,6 @@
         </is>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
   </sheetData>
   <autoFilter ref="$A$2:$F$47"/>
   <mergeCells count="1">
@@ -5048,7 +5914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5065,11 +5931,11 @@
           <t>📊 KPI MỤC TIÊU &amp; CHECKLIST TRACKING</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="3" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -5362,9 +6228,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -5392,9 +6258,9 @@
           <t>0</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>⬜ Chưa bắt đầu</t>
+      <c r="E12" s="43" t="inlineStr">
+        <is>
+          <t>✅ Hoàn thành</t>
         </is>
       </c>
       <c r="F12" s="10" t="inlineStr">
@@ -5493,7 +6359,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="35" customHeight="1">
       <c r="A17" s="33" t="n"/>
       <c r="B17" s="33" t="inlineStr">
@@ -6166,63 +7031,6 @@
       </c>
       <c r="F42" s="10" t="n"/>
     </row>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
@@ -6237,7 +7045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J199"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8854,141 +9662,6 @@
       </c>
       <c r="J64" s="10" t="n"/>
     </row>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
-    <row r="80"/>
-    <row r="81"/>
-    <row r="82"/>
-    <row r="83"/>
-    <row r="84"/>
-    <row r="85"/>
-    <row r="86"/>
-    <row r="87"/>
-    <row r="88"/>
-    <row r="89"/>
-    <row r="90"/>
-    <row r="91"/>
-    <row r="92"/>
-    <row r="93"/>
-    <row r="94"/>
-    <row r="95"/>
-    <row r="96"/>
-    <row r="97"/>
-    <row r="98"/>
-    <row r="99"/>
-    <row r="100"/>
-    <row r="101"/>
-    <row r="102"/>
-    <row r="103"/>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
   </sheetData>
   <autoFilter ref="$A$1:$J$47"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>